<commit_message>
US-051: plantilla de productos — el cliente define sus propias categorías
El cliente no usa nuestras categorías. Ahora la plantilla tiene una hoja
"Categorias" (paso 1) donde ingresa SUS categorías, y el dropdown de Categoría
en la hoja "Productos" lee esa lista (=Categorias!A2:A201), no un catálogo fijo.
El ISV queda fijo (estándar). Instrucciones reescritas en 2 pasos.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plantillas/plantilla_productos.xlsx
+++ b/docs/plantillas/plantilla_productos.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Listas" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet name="Productos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Categorias" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Productos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -486,9 +487,9 @@
       <c r="A4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Llená la hoja "Productos" (una fila por producto). Las filas en gris claro son EJEMPLOS: borralas o reemplazalas.</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>IMPORTANTE: este archivo tiene DOS pasos en este orden:</t>
         </is>
       </c>
     </row>
@@ -498,95 +499,126 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>COLUMNAS:</t>
+          <t>PASO 1 — Hoja "Categorias":</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>• Nombre *  (obligatorio): nombre del producto tal como aparecerá en facturas y catálogo.</t>
+          <t>• Ingresá PRIMERO todas TUS categorías (una por fila, en la columna 'Categoria').</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>• Categoria *  (obligatorio): elegí una de la lista desplegable. Si falta una categoría, avisanos para agregarla.</t>
+          <t>• Usá tus propios nombres de categoría — no hay una lista fija del sistema.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>• Impuesto (ISV) *  (obligatorio): Exectos (0%) = exonerado, Basicos (15%), Lujo (18%). Elegí de la lista.</t>
+          <t>• Las filas en gris son ejemplos: borralas y poné las tuyas.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>• Precio de venta *  (obligatorio): precio al público, en Lempiras, CON impuesto incluido. Solo números (ej. 25.00).</t>
-        </is>
-      </c>
+      <c r="A11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>• Codigo de barras  (opcional): si el producto tiene código de barras escaneable.</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>PASO 2 — Hoja "Productos" (una fila por producto):</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>• Codigo alterno  (opcional): código interno/SKU si manejás uno.</t>
+          <t>• Nombre *  (obligatorio): nombre del producto tal como aparecerá en facturas y catálogo.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr"/>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>• Categoria *  (obligatorio): elegí del desplegable — solo aparecen las categorías que cargaste en el PASO 1.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>REGLAS:</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>• Impuesto (ISV) *  (obligatorio): Exectos (0%) = exonerado, Basicos (15%), Lujo (18%). Elegí del desplegable.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>• No cambies los encabezados ni el orden de las columnas.</t>
+          <t>• Precio de venta *  (obligatorio): precio al público, en Lempiras, CON impuesto incluido. Solo números (ej. 25.00).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>• No dejes filas vacías en medio de los datos.</t>
+          <t>• Codigo de barras  (opcional): si el producto tiene código de barras escaneable.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>• Categoría e Impuesto deben venir SIEMPRE de la lista desplegable (validación activada).</t>
+          <t>• Codigo alterno  (opcional): código interno/SKU si manejás uno.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>• El precio incluye el ISV (el sistema calcula el desglose automáticamente).</t>
-        </is>
-      </c>
+      <c r="A19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>REGLAS:</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>• Cargá las categorías ANTES de los productos (el desplegable de Categoría se llena desde la hoja 'Categorias').</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>• No cambies los encabezados ni el orden de las columnas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>• No dejes filas vacías en medio de los datos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>• El precio incluye el ISV (el sistema calcula el desglose automáticamente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Cuando termines, guardá el archivo y envialo para la carga. Soporta varios cientos de productos por archivo.</t>
         </is>
@@ -603,17 +635,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Categorias</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
           <t>Impuestos</t>
         </is>
       </c>
@@ -621,11 +648,6 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ACCES</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
           <t>Exectos (0%)</t>
         </is>
       </c>
@@ -633,11 +655,6 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BEBE</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
           <t>Basicos (15%)</t>
         </is>
       </c>
@@ -645,173 +662,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BEBID</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
           <t>Lujo (18%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BOLSO</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CABELLO</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>COSTURA</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CUIDADO PERSONAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>DECOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ELECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ELECTRONICA</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>FERRE</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>FIEST</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>GOLOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>HOGAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>JOYERIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>JUGUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>MEDIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>OTROS</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>REGAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>RODA</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>ROPA</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>SEGUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>SERVI</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>UTIL</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Varios</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>ZAPAT</t>
         </is>
       </c>
     </row>
@@ -821,6 +672,65 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Categoria *</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>ABARROTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>BEBIDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>LIMPIEZA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>CUIDADO PERSONAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -877,7 +787,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>BEBID</t>
+          <t>BEBIDAS</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -924,32 +834,32 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Medicamento generico</t>
+          <t>Jabon de tocador</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>MEDIC</t>
+          <t>CUIDADO PERSONAL</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Exectos (0%)</t>
+          <t>Basicos (15%)</t>
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>45.5</v>
+        <v>18.5</v>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="B2:B604" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista." promptTitle="Ayuda" prompt="Seleccioná la categoría del producto." type="list">
-      <formula1>=Listas!$A$2:$A$27</formula1>
+    <dataValidation sqref="B2:B604" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista." promptTitle="Ayuda" prompt="Elegí una categoría de las que cargaste en la hoja 'Categorias'." type="list">
+      <formula1>=Categorias!$A$2:$A$201</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C604" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista." promptTitle="Ayuda" prompt="Seleccioná el ISV que aplica." type="list">
-      <formula1>=Listas!$B$2:$B$4</formula1>
+      <formula1>=Listas!$A$2:$A$4</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D604" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Precio inválido" error="El precio debe ser un número mayor o igual a 0." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
docs: decisiones Fase 2/3 de stock reservado + US-115..119 (Sprint 11)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019idpM4ouGHkvAv9tr79Qv2
</commit_message>
<xml_diff>
--- a/docs/plantillas/plantilla_productos.xlsx
+++ b/docs/plantillas/plantilla_productos.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -565,60 +565,67 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>• Codigo de barras  (opcional): si el producto tiene código de barras escaneable.</t>
+          <t>• Precio de costo  (opcional): lo que te cuesta el producto (precio de compra), en Lempiras. Solo números (ej. 18.00). Se usa para calcular el margen y en los reportes de inventario; si no lo manejás, dejalo vacío.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>• Codigo de barras  (opcional): si el producto tiene código de barras escaneable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t>• Codigo alterno  (opcional): código interno/SKU si manejás uno.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>REGLAS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>• Cargá las categorías ANTES de los productos (el desplegable de Categoría se llena desde la hoja 'Categorias').</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>• No cambies los encabezados ni el orden de las columnas.</t>
+          <t>• Cargá las categorías ANTES de los productos (el desplegable de Categoría se llena desde la hoja 'Categorias').</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>• No dejes filas vacías en medio de los datos.</t>
+          <t>• No cambies los encabezados ni el orden de las columnas.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t>• No dejes filas vacías en medio de los datos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t>• El precio incluye el ISV (el sistema calcula el desglose automáticamente).</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Cuando termines, guardá el archivo y envialo para la carga. Soporta varios cientos de productos por archivo.</t>
         </is>
@@ -736,15 +743,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -770,10 +778,15 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
+          <t>Precio de costo</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>Codigo de barras</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Codigo alterno</t>
         </is>
@@ -798,12 +811,15 @@
       <c r="D2" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>7501055300013</t>
         </is>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="G2" s="5" t="n">
         <v>1001</v>
       </c>
     </row>
@@ -826,8 +842,11 @@
       <c r="D3" s="5" t="n">
         <v>180</v>
       </c>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="n">
+      <c r="E3" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="n">
         <v>1002</v>
       </c>
     </row>
@@ -852,9 +871,10 @@
       </c>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="B2:B604" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista." promptTitle="Ayuda" prompt="Elegí una categoría de las que cargaste en la hoja 'Categorias'." type="list">
       <formula1>=Categorias!$A$2:$A$201</formula1>
     </dataValidation>
@@ -864,6 +884,9 @@
     <dataValidation sqref="D2:D604" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Precio inválido" error="El precio debe ser un número mayor o igual a 0." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
+    <dataValidation sqref="E2:E604" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Costo inválido" error="El costo debe ser un número mayor o igual a 0 (o dejarse vacío)." type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>